<commit_message>
5/28 system almost ompleted
</commit_message>
<xml_diff>
--- a/static.xlsx
+++ b/static.xlsx
@@ -4,6 +4,9 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="F1" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="F2" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="O1" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="O5M" sheetId="4" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,21 +14,258 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
-  <si>
-    <t>test1</t>
-  </si>
-  <si>
-    <t>test2</t>
-  </si>
-  <si>
-    <t>test3</t>
-  </si>
-  <si>
-    <t>test4</t>
-  </si>
-  <si>
-    <t>test5</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="84">
+  <si>
+    <t>fff1</t>
+  </si>
+  <si>
+    <t>fff2</t>
+  </si>
+  <si>
+    <t>fff3</t>
+  </si>
+  <si>
+    <t>fff4</t>
+  </si>
+  <si>
+    <t>fff5</t>
+  </si>
+  <si>
+    <t>fff6</t>
+  </si>
+  <si>
+    <t>fff7</t>
+  </si>
+  <si>
+    <t>fff8</t>
+  </si>
+  <si>
+    <t>fff9</t>
+  </si>
+  <si>
+    <t>fff10</t>
+  </si>
+  <si>
+    <t>fff11</t>
+  </si>
+  <si>
+    <t>fff12</t>
+  </si>
+  <si>
+    <t>fff13</t>
+  </si>
+  <si>
+    <t>fff14</t>
+  </si>
+  <si>
+    <t>fff15</t>
+  </si>
+  <si>
+    <t>fff16</t>
+  </si>
+  <si>
+    <t>fff17</t>
+  </si>
+  <si>
+    <t>fff18</t>
+  </si>
+  <si>
+    <t>fff19</t>
+  </si>
+  <si>
+    <t>fff20</t>
+  </si>
+  <si>
+    <t>fff21</t>
+  </si>
+  <si>
+    <t>fffff_1</t>
+  </si>
+  <si>
+    <t>ffff_2</t>
+  </si>
+  <si>
+    <t>fffff_2</t>
+  </si>
+  <si>
+    <t>ffff_3</t>
+  </si>
+  <si>
+    <t>fffff_3</t>
+  </si>
+  <si>
+    <t>ffff_4</t>
+  </si>
+  <si>
+    <t>fffff_4</t>
+  </si>
+  <si>
+    <t>ffff_5</t>
+  </si>
+  <si>
+    <t>fffff_5</t>
+  </si>
+  <si>
+    <t>ffff_6</t>
+  </si>
+  <si>
+    <t>fffff_6</t>
+  </si>
+  <si>
+    <t>ffff_7</t>
+  </si>
+  <si>
+    <t>fffff_7</t>
+  </si>
+  <si>
+    <t>ffff_8</t>
+  </si>
+  <si>
+    <t>fffff_8</t>
+  </si>
+  <si>
+    <t>ffff_9</t>
+  </si>
+  <si>
+    <t>fffff_9</t>
+  </si>
+  <si>
+    <t>ffff_10</t>
+  </si>
+  <si>
+    <t>fffff_10</t>
+  </si>
+  <si>
+    <t>ffff_11</t>
+  </si>
+  <si>
+    <t>fffff_11</t>
+  </si>
+  <si>
+    <t>oo1</t>
+  </si>
+  <si>
+    <t>oo2</t>
+  </si>
+  <si>
+    <t>oo3</t>
+  </si>
+  <si>
+    <t>oo4</t>
+  </si>
+  <si>
+    <t>oo5</t>
+  </si>
+  <si>
+    <t>oo6</t>
+  </si>
+  <si>
+    <t>oo7</t>
+  </si>
+  <si>
+    <t>oo8</t>
+  </si>
+  <si>
+    <t>oo9</t>
+  </si>
+  <si>
+    <t>oo10</t>
+  </si>
+  <si>
+    <t>oo11</t>
+  </si>
+  <si>
+    <t>oo12</t>
+  </si>
+  <si>
+    <t>oo13</t>
+  </si>
+  <si>
+    <t>oo14</t>
+  </si>
+  <si>
+    <t>oo15</t>
+  </si>
+  <si>
+    <t>oo16</t>
+  </si>
+  <si>
+    <t>oo17</t>
+  </si>
+  <si>
+    <t>oo18</t>
+  </si>
+  <si>
+    <t>oo19</t>
+  </si>
+  <si>
+    <t>oo20</t>
+  </si>
+  <si>
+    <t>oo21</t>
+  </si>
+  <si>
+    <t>o55_1</t>
+  </si>
+  <si>
+    <t>o55_2</t>
+  </si>
+  <si>
+    <t>o55_3</t>
+  </si>
+  <si>
+    <t>o55_4</t>
+  </si>
+  <si>
+    <t>o55_5</t>
+  </si>
+  <si>
+    <t>o55_6</t>
+  </si>
+  <si>
+    <t>o55_7</t>
+  </si>
+  <si>
+    <t>o55_8</t>
+  </si>
+  <si>
+    <t>o55_9</t>
+  </si>
+  <si>
+    <t>o55_10</t>
+  </si>
+  <si>
+    <t>o55_11</t>
+  </si>
+  <si>
+    <t>o55_12</t>
+  </si>
+  <si>
+    <t>o55_13</t>
+  </si>
+  <si>
+    <t>o55_14</t>
+  </si>
+  <si>
+    <t>o55_15</t>
+  </si>
+  <si>
+    <t>o55_16</t>
+  </si>
+  <si>
+    <t>o55_17</t>
+  </si>
+  <si>
+    <t>o55_18</t>
+  </si>
+  <si>
+    <t>o55_19</t>
+  </si>
+  <si>
+    <t>o55_20</t>
+  </si>
+  <si>
+    <t>o55_21</t>
   </si>
 </sst>
 </file>
@@ -75,6 +315,18 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -323,6 +575,674 @@
         <v>4</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1">
+        <v>7.0</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1">
+        <v>9.0</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1">
+        <v>11.0</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1">
+        <v>12.0</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1">
+        <v>14.0</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1">
+        <v>15.0</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1">
+        <v>16.0</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1">
+        <v>19.0</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1">
+        <v>20.0</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1">
+        <v>21.0</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1">
+        <v>7.0</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1">
+        <v>9.0</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1">
+        <v>11.0</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1">
+        <v>12.0</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1">
+        <v>14.0</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1">
+        <v>15.0</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1">
+        <v>16.0</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1">
+        <v>19.0</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1">
+        <v>20.0</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1">
+        <v>21.0</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1">
+        <v>7.0</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1">
+        <v>9.0</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1">
+        <v>11.0</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1">
+        <v>12.0</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1">
+        <v>14.0</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1">
+        <v>15.0</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1">
+        <v>16.0</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1">
+        <v>19.0</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1">
+        <v>20.0</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1">
+        <v>21.0</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1">
+        <v>1.0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1">
+        <v>2.0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1">
+        <v>3.0</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1">
+        <v>4.0</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1">
+        <v>5.0</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1">
+        <v>6.0</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1">
+        <v>7.0</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1">
+        <v>8.0</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1">
+        <v>9.0</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1">
+        <v>10.0</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1">
+        <v>11.0</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1">
+        <v>12.0</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1">
+        <v>14.0</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1">
+        <v>15.0</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1">
+        <v>16.0</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1">
+        <v>17.0</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1">
+        <v>18.0</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1">
+        <v>19.0</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1">
+        <v>20.0</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1">
+        <v>21.0</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>83</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>